<commit_message>
Add APP environment files and update workbook
Adds new APP teaching assets (`prostredi.png` and `prostredni.xlsx`) and updates `vyuka.xlsx` to include the latest lesson content.
</commit_message>
<xml_diff>
--- a/Teorie/2.IT/APP/vyuka.xlsx
+++ b/Teorie/2.IT/APP/vyuka.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\it-martinsramek\Downloads\SCMSD-IT-Martin-Sramek\Teorie\2.IT\APP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://scmsd-my.sharepoint.com/personal/it-martinsramek_stredniskola_com/Documents/Plocha/SCMSD-IT-Martin-Sramek/Teorie/2.IT/APP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADF7D94A-D570-4815-AB57-C20EE0AF4DA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{ADF7D94A-D570-4815-AB57-C20EE0AF4DA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4845B5F4-24F4-4026-9625-D3EA77E71A06}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{C7735200-00CF-4C48-B66D-CD3C1184F066}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C7735200-00CF-4C48-B66D-CD3C1184F066}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
@@ -276,6 +276,56 @@
         </a:p>
       </xdr:txBody>
     </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>438150</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>149305</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>162367</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Obrázek 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C37E60B-73A0-8B57-CAA1-F04EDCBB0B8B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2266950" y="1343025"/>
+          <a:ext cx="8245555" cy="5105842"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>

</xml_diff>